<commit_message>
LR sweep complete: best lr=1e-5 → test/abs_rel=0.0478 (vs 0.0503 @ lr=1e-4)
Sweep results (test split, 25 epochs, KB-crop 350x1218 protocol):
  lr=5e-5: abs_rel=0.0493 rmse=2.117 d1=0.9791
  lr=3e-5: abs_rel=0.0484 rmse=2.158 d1=0.9795
  lr=1e-5: abs_rel=0.0478 rmse=2.026 d1=0.9821  <-- best abs_rel
  lr=5e-6: abs_rel=0.0484 rmse=2.013 d1=0.9825  <-- best rmse/d1
  lr=1e-6: abs_rel=0.0494 rmse=2.051 d1=0.9822

Best fine-tune lr = 1e-5 (small-lr sweet spot for a strong pretrained model).

Add scripts/eval_official.{py,bsub}: standalone paper-protocol evaluator
(short-side 518 + Garg crop + 80 m cap) for apples-to-apples comparison
with published KITTI Eigen numbers.
</commit_message>
<xml_diff>
--- a/experiments.xlsx
+++ b/experiments.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -706,6 +706,11 @@
           <t>2026-04-23 02:07:33</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-04-23 09:45:49</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>vitl</t>
@@ -755,6 +760,32 @@
         <is>
           <t>eigen_train/eigen_test</t>
         </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>/fs/scratch/rb-bd-dlp-rng-dl01-cr-tfx/driving/tfx-201/users/izi2sgh/quanjie/liren/depth-v3/training-for-depth-anything-v3/logs/depth_anything_v3/kitti_eigen_vitl_lr5e-5/checkpoints/epoch08-val_abs_rel0.0493.ckpt</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0.04929960891604424</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.1460516005754471</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2.117156028747559</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.07430016994476318</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.9790608286857605</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.9977505803108215</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.9994132518768311</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -785,7 +816,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -798,6 +829,11 @@
           <t>2026-04-23 02:08:05</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-04-23 09:46:38</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>vitl</t>
@@ -847,6 +883,32 @@
         <is>
           <t>eigen_train/eigen_test</t>
         </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>/fs/scratch/rb-bd-dlp-rng-dl01-cr-tfx/driving/tfx-201/users/izi2sgh/quanjie/liren/depth-v3/training-for-depth-anything-v3/logs/depth_anything_v3/kitti_eigen_vitl_lr3e-5/checkpoints/epoch08-val_abs_rel0.0484.ckpt</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0.04837790504097939</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.144591435790062</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2.157958507537842</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.07344570755958557</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.9794800281524658</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.9977172613143921</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.9994167685508728</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -877,7 +939,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -890,6 +952,11 @@
           <t>2026-04-23 02:58:33</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:35:51</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>vitl</t>
@@ -939,6 +1006,32 @@
         <is>
           <t>eigen_train/eigen_test</t>
         </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>/fs/scratch/rb-bd-dlp-rng-dl01-cr-tfx/driving/tfx-201/users/izi2sgh/quanjie/liren/depth-v3/training-for-depth-anything-v3/logs/depth_anything_v3/kitti_eigen_vitl_lr1e-5/checkpoints/epoch09-val_abs_rel0.0478.ckpt</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>0.04780921339988708</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.1327967047691345</v>
+      </c>
+      <c r="U5" t="n">
+        <v>2.025900840759277</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.07126437127590179</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.9821373224258423</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.9980424046516418</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.999569296836853</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -969,7 +1062,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -982,6 +1075,11 @@
           <t>2026-04-23 03:36:17</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:11:59</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>vitl</t>
@@ -1031,6 +1129,32 @@
         <is>
           <t>eigen_train/eigen_test</t>
         </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>/fs/scratch/rb-bd-dlp-rng-dl01-cr-tfx/driving/tfx-201/users/izi2sgh/quanjie/liren/depth-v3/training-for-depth-anything-v3/logs/depth_anything_v3/kitti_eigen_vitl_lr5e-6/checkpoints/epoch14-val_abs_rel0.0484.ckpt</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0.04838978499174118</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.131302997469902</v>
+      </c>
+      <c r="U6" t="n">
+        <v>2.01285719871521</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.07127462327480316</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.9825325012207031</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.998082160949707</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.9995735883712769</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1061,7 +1185,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1074,6 +1198,11 @@
           <t>2026-04-23 03:45:37</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-04-23 11:25:02</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>vitl</t>
@@ -1123,6 +1252,32 @@
         <is>
           <t>eigen_train/eigen_test</t>
         </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>/fs/scratch/rb-bd-dlp-rng-dl01-cr-tfx/driving/tfx-201/users/izi2sgh/quanjie/liren/depth-v3/training-for-depth-anything-v3/logs/depth_anything_v3/kitti_eigen_vitl_lr1e-6/checkpoints/epoch22-val_abs_rel0.0494.ckpt</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>0.04936592653393745</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.1350692957639694</v>
+      </c>
+      <c r="U7" t="n">
+        <v>2.051220178604126</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.07304090261459351</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.9822233915328979</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.997942328453064</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0.9995369911193848</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>

</xml_diff>